<commit_message>
resolution des conflits 21c7c64a395fa9ac810273673c267020206861ff
</commit_message>
<xml_diff>
--- a/ML-Entrees/ig/StructureDefinition-fr-lm-acte-imagerie.xlsx
+++ b/ML-Entrees/ig/StructureDefinition-fr-lm-acte-imagerie.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-14T07:59:58+00:00</t>
+    <t>2026-04-16T07:11:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -357,7 +357,7 @@
     <t>fr-lm-acte-imagerie.entree.administrationProduits</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-administration-produit-de-sante
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-dicom-medication-administration
 </t>
   </si>
   <si>
@@ -676,7 +676,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="83.87109375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="84.88671875" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>